<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.002-05 La sonnette argentée de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-05.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-05.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut faire ding au square avec la trottinette. Le guidon heurte le manteau bleu au crochet. Elle range la trottinette, enfile le manteau, sonne au square, rentre, raccroche.</t>
+          <t>Nina connaît l'entrée. Un éclat de sonnette cligne sur le métal froid. Elle veut ding au square du banc vide, maintenant. Elle roule sans le manteau : le guidon heurte le crochet, la manche cache l'éclat. Elle refuse de tirer les deux à la fois, pose la trottinette, prend le manteau. Au square, la sonnette reste muette. Elle refuse de foncer, retrouve l'éclat, fait ding. Le manteau rentre au crochet.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La trottinette s'appuie au mur. Sa sonnette est argentée. Une bande de soleil coupe les carreaux. Les chaussures de papa font une paire. Le square est juste en bas de la rue. Nina, tu as vu la sonnette ? Elle brille, papa. En ce moment, Nina touche le guidon. La sonnette est froide. Son manteau bleu attend au crochet. On va au square ? Oui. Avec la trottinette. Nina fait rouler la trottinette. Les roues font un bruit léger. Le guidon heurte le crochet. Le manteau bleu se balance. Oh. Le manteau a bougé. Pose la trottinette un moment. On prend le manteau d'abord. Nina pose la trottinette contre le mur. Elle prend son manteau bleu. Elle passe les manches. Le tissu est doux. Tu as le manteau ? Oui. On ouvre la porte ? Oui. Doucement. Papa ouvre la porte. L'air est frais. Ils sortent. Au square, Nina pousse la trottinette. Les roues chantent un peu. La sonnette fait ding, une fois. Ding ! Tu as le manteau bien mis ? Oui. J'ai chaud. Un banc est vide. Nina s'arrête un moment. Elle pose un pied par terre. Les feuilles du square sont sèches. Elles craquent sous la roue. Tu as entendu les feuilles ? Oui. Ça fait chh. Encore un ding ? Nina touche la sonnette. Ça fait ding encore. C'est l'heure de rentrer. Oui. On rentre. Ils rentrent. Nina raccroche le manteau au crochet. Le crochet est bas. Elle pose la trottinette contre le mur. Nina essuie un peu le guidon. La sonnette est froide sous le doigt. Tu as fini de poser la trottinette ? Oui. Contre le mur.</t>
+          <t>Une bande de soleil coupe les carreaux de l'entrée. Nina connaît cette entrée, le crochet, les bruits du carreau. Les chaussures de papa font une paire, près de la porte. La trottinette s'appuie au mur, un peu penchée. Un détail paraît nouveau, sur le métal. Sur la sonnette argentée, un éclat de sonnette cligne. Le métal est froid, presque blanc. Nina, tu vois l'éclat ? Il brille, papa. Je veux ding au square, maintenant ! Le square du banc vide est juste en bas de la rue. On y va, avec la trottinette. En ce moment, Nina saisit le guidon froid. Son manteau bleu attend au crochet, trop loin. Vite, le banc est vide ! Elle pousse la trottinette vers la porte. Les roues font un bruit léger, sur les carreaux. Le guidon heurte le crochet, dur. Le manteau bleu se balance, puis retombe. Une manche glisse sur la sonnette. L'éclat de sonnette disparaît sous le tissu. Oh. Il est parti ! Pose la trottinette un moment. Nina veut les deux, d'un coup. Elle tire le manteau, le guidon sous l'autre bras. La manche se tord, serrée. Le tissu refuse de venir. Ça reste coincé ! Elle tire plus fort. Le crochet penche, un peu. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à sa hauteur. Tu regardes le manteau ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La trottinette s'appuie au mur. Sa sonnette est argentée. Une bande de soleil coupe les carreaux. Les chaussures de papa font une paire. Le square est juste en bas de la rue. Nina, tu as vu la sonnette ? Elle brille, papa. En ce moment, Nina touche le guidon. La sonnette est froide. Son manteau bleu attend au crochet. On va au square ? Oui. Avec la trottinette. Nina fait rouler la trottinette. Les roues font un bruit léger. Le guidon heurte le crochet. Le manteau bleu se balance. Oh. Le manteau a bougé. Pose la trottinette un moment. On prend le manteau d'abord. Nina pose la trottinette contre le mur. Elle prend son manteau bleu. Elle passe les manches. Le tissu est doux. Tu as le manteau ? Oui. On ouvre la porte ? Oui. Doucement. Papa ouvre la porte. L'air est frais. Ils sortent. Au square, Nina pousse la trottinette. Les roues chantent un peu. La sonnette fait ding, une fois. Ding ! Tu as le manteau bien mis ? Oui. J'ai chaud. Un banc est vide. Nina s'arrête un moment. Elle pose un pied par terre. Les feuilles du square sont sèches. Elles craquent sous la roue. Tu as entendu les feuilles ? Oui. Ça fait chh. Encore un ding ? Nina touche la sonnette. Ça fait ding encore. C'est l'heure de rentrer. Oui. On rentre. Ils rentrent. Nina raccroche le manteau au crochet. Le crochet est bas. Elle pose la trottinette contre le mur. Nina essuie un peu le guidon. La sonnette est froide sous le doigt. Tu as fini de poser la trottinette ? Oui. Contre le mur.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une bande de soleil coupe les carreaux de l'entrée. Nina connaît cette entrée, le crochet, les bruits du carreau. Les chaussures de papa font une paire, près de la porte. La trottinette s'appuie au mur, un peu penchée. Un détail paraît nouveau, sur le métal. Sur la sonnette argentée, un &lt;emphasis level="moderate"&gt;éclat de sonnette&lt;/emphasis&gt; cligne. Le métal est froid, presque blanc. Nina, tu vois l'éclat ? Il brille, papa. Je veux ding au square, maintenant ! Le square du banc vide est juste en bas de la rue. On y va, avec la trottinette. En ce moment, Nina saisit le guidon froid. Son manteau bleu attend au crochet, trop loin. Vite, le banc est vide ! Elle pousse la trottinette vers la porte. Les roues font un bruit léger, sur les carreaux. Le guidon heurte le crochet, dur. Le manteau bleu se balance, puis retombe. Une manche glisse sur la sonnette. L'éclat de sonnette disparaît sous le tissu. Oh. Il est parti ! Pose la trottinette un moment. Nina veut les deux, d'un coup. Elle tire le manteau, le guidon sous l'autre bras. La manche se tord, serrée. Le tissu refuse de venir. Ça reste coincé ! Elle tire plus fort. Le crochet penche, un peu. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à sa hauteur. Tu regardes le manteau ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Damien veut aller au square. Papa ouvre la porte de l'entrée. L'air est frais. Papa dit : avant de sortir, on prend le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Damien prend son manteau bleu. Il passe les manches. Le tissu est doux. Ils sortent. Au square, Damien pousse la trottinette. Les roues font un bruit léger. Puis ils rentrent. Papa dit : en rentrant, le manteau va à sa place. Damien raccroche le manteau au crochet. Le crochet est bas. Damien dit : manteau pour sortir. Manteau à sa place en rentrant. Papa sourit. Les chaussures restent près de la porte. [pause]</t>
+          <t>Une bande de soleil coupe les carreaux de l'entrée. Nina connaît cette entrée, le crochet, les bruits du carreau. Les chaussures de papa font une paire, près de la porte. La trottinette s'appuie au mur, un peu penchée. Un détail paraît nouveau, sur le métal. Sur la sonnette argentée, un &lt;emphasis&gt;éclat de sonnette&lt;/emphasis&gt; cligne. Le métal est froid, presque blanc. Nina, tu vois l'éclat ? Il brille, papa. Je veux ding au square, maintenant ! Le square du banc vide est juste en bas de la rue. On y va, avec la trottinette. En ce moment, Nina saisit le guidon froid. Son manteau bleu attend au crochet, trop loin. Vite, le banc est vide ! Elle pousse la trottinette vers la porte. Les roues font un bruit léger, sur les carreaux. Le guidon heurte le crochet, dur. Le manteau bleu se balance, puis retombe. Une manche glisse sur la sonnette. L'éclat de sonnette disparaît sous le tissu. Oh. Il est parti ! Pose la trottinette un moment. Nina veut les deux, d'un coup. Elle tire le manteau, le guidon sous l'autre bras. La manche se tord, serrée. Le tissu refuse de venir. Ça reste coincé ! Elle tire plus fort. Le crochet penche, un peu. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à sa hauteur. Tu regardes le manteau ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat de sonnette</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,72 +1326,48 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_ding_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La trottinette s'appuie au mur.
-narrateur|Sa sonnette est argentée.
-narrateur|Une bande de soleil coupe les carreaux.
-narrateur|Les chaussures de papa font une paire.
-narrateur|Le square est juste en bas de la rue.
-papa|Nina, tu as vu la sonnette ?
-enfant-f|Elle brille, papa.
-narrateur|En ce moment, Nina touche le guidon.
-narrateur|La sonnette est froide.
-narrateur|Son manteau bleu attend au crochet.
-enfant-f|On va au square ?
-papa|Oui.
-papa|Avec la trottinette.
-narrateur|Nina fait rouler la trottinette.
-narrateur|Les roues font un bruit léger.
-narrateur|Le guidon heurte le crochet.
-narrateur|Le manteau bleu se balance.
+          <t>narrateur|Une bande de soleil coupe les carreaux de l'entrée.
+narrateur|Nina connaît cette entrée, le crochet, les bruits du carreau.
+narrateur|Les chaussures de papa font une paire, près de la porte.
+narrateur|La trottinette s'appuie au mur, un peu penchée.
+narrateur|Un détail paraît nouveau, sur le métal.
+narrateur|Sur la sonnette argentée, un éclat de sonnette cligne.
+narrateur|Le métal est froid, presque blanc.
+papa|Nina, tu vois l'éclat ?
+enfant-f|Il brille, papa.
+enfant-f|Je veux ding au square, maintenant !
+narrateur|Le square du banc vide est juste en bas de la rue.
+papa|On y va, avec la trottinette.
+narrateur|En ce moment, Nina saisit le guidon froid.
+narrateur|Son manteau bleu attend au crochet, trop loin.
+enfant-f|Vite, le banc est vide !
+narrateur|Elle pousse la trottinette vers la porte.
+narrateur|Les roues font un bruit léger, sur les carreaux.
+narrateur|Le guidon heurte le crochet, dur.
+narrateur|Le manteau bleu se balance, puis retombe.
+narrateur|Une manche glisse sur la sonnette.
+narrateur|L'éclat de sonnette disparaît sous le tissu.
 enfant-f|Oh.
-enfant-f|Le manteau a bougé.
+enfant-f|Il est parti !
 papa|Pose la trottinette un moment.
-papa|On prend le manteau d'abord.
-narrateur|Nina pose la trottinette contre le mur.
-narrateur|Elle prend son manteau bleu.
-narrateur|Elle passe les manches.
-narrateur|Le tissu est doux.
-papa|Tu as le manteau ?
-enfant-f|Oui.
-papa|On ouvre la porte ?
-enfant-f|Oui.
-enfant-f|Doucement.
-narrateur|Papa ouvre la porte.
-narrateur|L'air est frais.
-narrateur|Ils sortent.
-narrateur|Au square, Nina pousse la trottinette.
-narrateur|Les roues chantent un peu.
-narrateur|La sonnette fait ding, une fois.
-enfant-f|Ding !
-papa|Tu as le manteau bien mis ?
-enfant-f|Oui.
-enfant-f|J'ai chaud.
-narrateur|Un banc est vide.
-narrateur|Nina s'arrête un moment.
-narrateur|Elle pose un pied par terre.
-narrateur|Les feuilles du square sont sèches.
-narrateur|Elles craquent sous la roue.
-papa|Tu as entendu les feuilles ?
-enfant-f|Oui.
-enfant-f|Ça fait chh.
-papa|Encore un ding ?
-narrateur|Nina touche la sonnette.
-narrateur|Ça fait ding encore.
-papa|C'est l'heure de rentrer.
-enfant-f|Oui.
-enfant-f|On rentre.
-narrateur|Ils rentrent.
-narrateur|Nina raccroche le manteau au crochet.
-narrateur|Le crochet est bas.
-narrateur|Elle pose la trottinette contre le mur.
-narrateur|Nina essuie un peu le guidon.
-narrateur|La sonnette est froide sous le doigt.
-papa|Tu as fini de poser la trottinette ?
-enfant-f|Oui.
-enfant-f|Contre le mur.</t>
+narrateur|Nina veut les deux, d'un coup.
+narrateur|Elle tire le manteau, le guidon sous l'autre bras.
+narrateur|La manche se tord, serrée.
+narrateur|Le tissu refuse de venir.
+enfant-f|Ça reste coincé !
+narrateur|Elle tire plus fort.
+narrateur|Le crochet penche, un peu.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à sa hauteur.
+papa|Tu regardes le manteau ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1423,17 +1399,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Nina ?</t>
+          <t>Nina prépare la sortie. Le manteau bleu attend au crochet. Avant de sortir, que prend Nina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina prépare la sortie. Le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; bleu attend au crochet. Avant de sortir, que prend Nina ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Avant de &lt;emphasis&gt;sortir&lt;/emphasis&gt;, que prend Damien ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina prépare la sortie. Le &lt;emphasis&gt;manteau&lt;/emphasis&gt; bleu attend au crochet. Avant de sortir, que prend Nina ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1496,7 +1472,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1507,7 +1483,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1522,38 +1498,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>sortir</t>
+          <t>manteau</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1568,22 +1544,24 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=avant_de_sortir_le_manteau; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de sortir, que prend Nina ?</t>
+          <t>narrateur|Nina prépare la sortie.
+narrateur|Le manteau bleu attend au crochet.
+narrateur|Avant de sortir, que prend Nina ?</t>
         </is>
       </c>
     </row>
@@ -1610,17 +1588,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina a pris le manteau bleu. Elle l'a mis pour le square. Elle a poussé la trottinette. La sonnette a fait ding. En rentrant, elle a raccroché. Tu as pris le manteau pour sortir. Il est à sa place. Oui. Près de la trottinette.</t>
+          <t>Nina refuse de tirer plus fort. Elle pose la trottinette contre le mur. Les roues s'arrêtent, nettes. Je pose le guidon. Elle soulève la manche, lente. Sous le tissu, l'éclat de sonnette cligne. Il est là, papa. Tu le vois, toi ? Oui, sur la sonnette. Nina prend son manteau bleu. Elle passe une manche, puis l'autre. Le tissu est doux, un peu frais. Tu as le manteau ? Oui, papa. Le crochet reste vide, bas. La sonnette est libre, froide. Merci, Nina. On ouvre la porte ? Oui. Papa ouvre la porte. L'air est frais, un peu vif. Ils sortent vers le square du banc vide. Nina pose la main sur le guidon. Le métal reste froid sous le doigt. On y va. Oui, l'air est frais.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina a pris le manteau bleu. Elle l'a mis pour le square. Elle a poussé la trottinette. La sonnette a fait ding. En rentrant, elle a raccroché. Tu as pris le manteau pour sortir. Il est à sa place. Oui. Près de la trottinette.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina refuse de tirer plus fort. Elle pose la trottinette contre le mur. Les roues s'arrêtent, nettes. Je pose le guidon. Elle soulève la manche, lente. Sous le tissu, l'éclat de sonnette cligne. Il est là, papa. Tu le vois, toi ? Oui, sur la sonnette. Nina prend son &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; bleu. Elle passe une manche, puis l'autre. Le tissu est doux, un peu frais. Tu as le manteau ? Oui, papa. Le crochet reste vide, bas. La sonnette est libre, froide. Merci, Nina. On ouvre la porte ? Oui. Papa ouvre la porte. L'air est frais, un peu vif. Ils sortent vers le square du banc vide. Nina pose la main sur le guidon. Le métal reste froid sous le doigt. On y va. Oui, l'air est frais.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Damien a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt; pour sortir. En rentrant, il l'a raccroché. [pause]</t>
+          <t>Nina refuse de tirer plus fort. Elle pose la trottinette contre le mur. Les roues s'arrêtent, nettes. Je pose le guidon. Elle soulève la manche, lente. Sous le tissu, l'éclat de sonnette cligne. Il est là, papa. Tu le vois, toi ? Oui, sur la sonnette. Nina prend son &lt;emphasis&gt;manteau&lt;/emphasis&gt; bleu. Elle passe une manche, puis l'autre. Le tissu est doux, un peu frais. Tu as le manteau ? Oui, papa. Le crochet reste vide, bas. La sonnette est libre, froide. Merci, Nina. On ouvre la porte ? Oui. Papa ouvre la porte. L'air est frais, un peu vif. Ils sortent vers le square du banc vide. Nina pose la main sur le guidon. Le métal reste froid sous le doigt. On y va. Oui, l'air est frais. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1678,7 +1656,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1715,16 +1693,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1749,20 +1727,42 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=fierté_calme; intensite=1; destinataire=enfant; sous_texte=elle_prend_le_manteau_sans_foncer; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina a pris le manteau bleu.
-narrateur|Elle l'a mis pour le square.
-narrateur|Elle a poussé la trottinette.
-narrateur|La sonnette a fait ding.
-narrateur|En rentrant, elle a raccroché.
-papa|Tu as pris le manteau pour sortir.
-enfant-f|Il est à sa place.
-papa|Oui.
-papa|Près de la trottinette.</t>
+          <t>narrateur|Nina refuse de tirer plus fort.
+narrateur|Elle pose la trottinette contre le mur.
+narrateur|Les roues s'arrêtent, nettes.
+enfant-f|Je pose le guidon.
+narrateur|Elle soulève la manche, lente.
+narrateur|Sous le tissu, l'éclat de sonnette cligne.
+enfant-f|Il est là, papa.
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur la sonnette.
+narrateur|Nina prend son manteau bleu.
+narrateur|Elle passe une manche, puis l'autre.
+narrateur|Le tissu est doux, un peu frais.
+papa|Tu as le manteau ?
+enfant-f|Oui, papa.
+narrateur|Le crochet reste vide, bas.
+narrateur|La sonnette est libre, froide.
+papa|Merci, Nina.
+papa|On ouvre la porte ?
+enfant-f|Oui.
+narrateur|Papa ouvre la porte.
+narrateur|L'air est frais, un peu vif.
+narrateur|Ils sortent vers le square du banc vide.
+narrateur|Nina pose la main sur le guidon.
+narrateur|Le métal reste froid sous le doigt.
+enfant-f|On y va.
+papa|Oui, l'air est frais.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,porte</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1789,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina pose ses chaussures. Papa ferme la porte. La bande de soleil a bougé. Tu as fini de poser tes chaussures ? Oui, papa. La sonnette est silencieuse. Le manteau bleu reste au crochet. On reste un peu à la maison. La trottinette attend. Oui. Et le manteau aussi.</t>
+          <t>Au square, Nina pousse la trottinette. Les roues chantent un peu, sur le gravier. Un banc est vide, au soleil. Ding, maintenant ! Elle appuie trop fort, d'un coup. La sonnette reste muette. Elle ne veut pas. Les feuilles du square sont sèches. Elles font chh, sous la roue. Nina veut appuyer plus fort. Elle refuse de foncer. Attends, je regarde. Papa attend, sans parler. Elle observe la sonnette, puis le square. Le métal est tourné, de travers. Sur l'autre face, un éclat de sonnette cligne. C'est celui de l'entrée. Tu le vois, au square ? Oui, il s'était caché. Nina tourne le métal, sans brusquer. L'éclat de sonnette revient face au soleil. Elle appuie, légère. Ça fait ding, une fois. Ding ! Tu l'as fait sonner ? Oui, elle était tournée. Le banc vide reste au soleil. Nina pose un pied par terre. On rentre, Nina ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina pose ses chaussures. Papa ferme la porte. La bande de soleil a bougé. Tu as fini de poser tes chaussures ? Oui, papa. La sonnette est silencieuse. Le manteau bleu reste au crochet. On reste un peu à la maison. La trottinette attend. Oui. Et le manteau aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au square, Nina pousse la trottinette. Les roues chantent un peu, sur le gravier. Un banc est vide, au soleil. Ding, maintenant ! Elle appuie trop fort, d'un coup. La sonnette reste muette. Elle ne veut pas. Les feuilles du square sont sèches. Elles font chh, sous la roue. Nina veut appuyer plus fort. Elle refuse de foncer. Attends, je regarde. Papa attend, sans parler. Elle observe la sonnette, puis le square. Le métal est tourné, de travers. Sur l'autre face, un &lt;emphasis level="moderate"&gt;éclat de sonnette&lt;/emphasis&gt; cligne. C'est celui de l'entrée. Tu le vois, au square ? Oui, il s'était caché. Nina tourne le métal, sans brusquer. L'éclat de sonnette revient face au soleil. Elle appuie, légère. Ça fait ding, une fois. Ding ! Tu l'as fait sonner ? Oui, elle était tournée. Le banc vide reste au soleil. Nina pose un pied par terre. On rentre, Nina ? Oui, papa.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Damien pose ses chaussures. Papa ferme la porte. [pause]</t>
+          <t>&lt;low-pitch&gt;Au square, Nina pousse la trottinette. Les roues chantent un peu, sur le gravier. Un banc est vide, au soleil. Ding, maintenant ! Elle appuie trop fort, d'un coup. La sonnette reste muette. Elle ne veut pas. Les feuilles du square sont sèches. Elles font chh, sous la roue. Nina veut appuyer plus fort. Elle refuse de foncer. Attends, je regarde. Papa attend, sans parler. Elle observe la sonnette, puis le square. Le métal est tourné, de travers. Sur l'autre face, un &lt;emphasis&gt;éclat de sonnette&lt;/emphasis&gt; cligne. C'est celui de l'entrée. Tu le vois, au square ? Oui, il s'était caché. Nina tourne le métal, sans brusquer. L'éclat de sonnette revient face au soleil. Elle appuie, légère. Ça fait ding, une fois. Ding ! Tu l'as fait sonner ? Oui, elle était tournée. Le banc vide reste au soleil. Nina pose un pied par terre. On rentre, Nina ? Oui, papa.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1854,22 +1854,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1878,28 +1882,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de sonnette</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1908,34 +1916,62 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina pose ses chaussures.
-narrateur|Papa ferme la porte.
-narrateur|La bande de soleil a bougé.
-papa|Tu as fini de poser tes chaussures ?
-enfant-f|Oui, papa.
-narrateur|La sonnette est silencieuse.
-narrateur|Le manteau bleu reste au crochet.
-papa|On reste un peu à la maison.
-enfant-f|La trottinette attend.
-papa|Oui.
-papa|Et le manteau aussi.</t>
+          <t>narrateur|Au square, Nina pousse la trottinette.
+narrateur|Les roues chantent un peu, sur le gravier.
+narrateur|Un banc est vide, au soleil.
+enfant-f|Ding, maintenant !
+narrateur|Elle appuie trop fort, d'un coup.
+narrateur|La sonnette reste muette.
+enfant-f|Elle ne veut pas.
+narrateur|Les feuilles du square sont sèches.
+narrateur|Elles font chh, sous la roue.
+narrateur|Nina veut appuyer plus fort.
+narrateur|Elle refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Elle observe la sonnette, puis le square.
+narrateur|Le métal est tourné, de travers.
+narrateur|Sur l'autre face, un éclat de sonnette cligne.
+enfant-f|C'est celui de l'entrée.
+papa|Tu le vois, au square ?
+enfant-f|Oui, il s'était caché.
+narrateur|Nina tourne le métal, sans brusquer.
+narrateur|L'éclat de sonnette revient face au soleil.
+narrateur|Elle appuie, légère.
+narrateur|Ça fait ding, une fois.
+enfant-f|Ding !
+papa|Tu l'as fait sonner ?
+enfant-f|Oui, elle était tournée.
+narrateur|Le banc vide reste au soleil.
+narrateur|Nina pose un pied par terre.
+papa|On rentre, Nina ?
+enfant-f|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>sonnette,feuilles</t>
         </is>
       </c>
     </row>
@@ -1962,17 +1998,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai fait ding au square. J'avais le manteau. Bravo, Nina. La sonnette argentée attend contre le mur.</t>
+          <t>Ils rentrent dans l'entrée. Papa ferme la porte. Nina raccroche le manteau au crochet. Il est à sa place. Le crochet est bas, à sa hauteur. Elle pose la trottinette contre le mur. Tu as fini de poser tes chaussures ? Oui, papa. La bande de soleil a bougé, sur les carreaux. J'ai fait ding au banc. Oui, tu l'as fait. La sonnette argentée attend contre le mur. L'éclat de sonnette reste, pâle, sur le métal.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai fait ding au square. J'avais le manteau. Bravo, Nina. La sonnette argentée attend contre le mur.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent dans l'entrée. Papa ferme la porte. Nina raccroche le manteau au crochet. Il est à sa place. Le crochet est bas, à sa hauteur. Elle pose la trottinette contre le mur. Tu as fini de poser tes chaussures ? Oui, papa. La bande de soleil a bougé, sur les carreaux. J'ai fait ding au banc. Oui, tu l'as fait. La sonnette argentée attend contre le mur. L'&lt;emphasis level="moderate"&gt;éclat de sonnette&lt;/emphasis&gt; reste, pâle, sur le métal.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent dans l'entrée. Papa ferme la porte. Nina raccroche le manteau au crochet. Il est à sa place. Le crochet est bas, à sa hauteur. Elle pose la trottinette contre le mur. Tu as fini de poser tes chaussures ? Oui, papa. La bande de soleil a bougé, sur les carreaux. J'ai fait ding au banc. Oui, tu l'as fait. La sonnette argentée attend contre le mur. L'&lt;emphasis&gt;éclat de sonnette&lt;/emphasis&gt; reste, pâle, sur le métal.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2019,7 +2055,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2027,7 +2063,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2039,12 +2075,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2053,17 +2089,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de sonnette</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2072,11 +2112,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2085,27 +2125,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_reste_sur_le_metal_le_manteau_au_crochet; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai fait ding au square.
-enfant-f|J'avais le manteau.
-papa|Bravo, Nina.
-narrateur|La sonnette argentée attend contre le mur.</t>
+          <t>narrateur|Ils rentrent dans l'entrée.
+narrateur|Papa ferme la porte.
+narrateur|Nina raccroche le manteau au crochet.
+enfant-f|Il est à sa place.
+narrateur|Le crochet est bas, à sa hauteur.
+narrateur|Elle pose la trottinette contre le mur.
+papa|Tu as fini de poser tes chaussures ?
+enfant-f|Oui, papa.
+narrateur|La bande de soleil a bougé, sur les carreaux.
+enfant-f|J'ai fait ding au banc.
+papa|Oui, tu l'as fait.
+narrateur|La sonnette argentée attend contre le mur.
+narrateur|L'éclat de sonnette reste, pâle, sur le métal.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2276,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>